<commit_message>
9.13: docs(deliverable): Launch 준비 xlsx 갱신 — 하드닝 이력 9.7~9.12 추가, 품질·설계 결정 시트 신설(muted 텍스트 WCAG AA 미달=설계 판단·#77·CSP script-src 후속)
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Launch 차단 - 사용자 필요" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Launch 하드닝 이력" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. 보안 감사" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. 품질·설계 결정" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3530,7 +3531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3712,6 +3713,138 @@
       <c r="D8" s="2" t="inlineStr">
         <is>
           <t>라이브 8/8</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Launch 준비 딜리버러블</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>요구/차단/하드닝 xlsx</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>보안 응답 헤더</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>HSTS·nosniff·X-Frame·Referrer·버전숨김</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>최소 CSP + 보안 감사</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>frame-ancestors·base-uri·object-src·CORS/쿠키/시크릿</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>E2E 무결</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>9.10</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>보안 감사 시트</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>SQL인젝션 전수(AST 0건) 등 10영역</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>9.11</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>플릿 동시실행 락</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>시드 손상 유발 충돌 방지</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>뮤테이션 검증</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>9.12</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>a11y: html lang</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>ko 하드코딩→실 로케일(en/ja/zh)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>라이브 확인</t>
         </is>
       </c>
     </row>
@@ -3980,4 +4113,108 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>상태</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>html lang 로케일</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>조치완료(9.12)</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>en/ja/zh 사용자에게 실 로케일 선언 — 라이브 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>색상 대비(muted 텍스트)</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>설계 결정 필요</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>주 텍스트 15:1(우수). --txt-mute #8B93A1 ≈3.2:1 은 WCAG AA 일반텍스트(4.5:1) 미달·큰텍스트(3:1) 통과. 의도적 약화 텍스트라 darken 은 시각 위계 변경 — 디자인 소유자 판단</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Head Type 목록(#77)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>결정 필요</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Freeze 6종 vs 코드 SYSTEM/TENANT 2종 — 권한 임계 필드</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>전체 CSP script-src</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>후속</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>현재 최소 CSP. script-src 는 Next 인라인 검증 후</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
9.26: docs: Launch 준비 딜리버러블 갱신 — 하드닝 9.14~9.25·검증 상태(SSR 60/60·플릿 105/105) 반영
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -520,7 +520,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -617,31 +617,31 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>전 화면 E2E 브라우저 스윕 (62화면·쓰기·결재·명령줄)</t>
+          <t>전 화면 로그인 SSR 렌더 스윕 (60화면·인증 200 무오류)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS 60/60</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>핵심 매출 파이프라인 (CPQ→BOM→치수→도면→단가→견적PDF)</t>
+          <t>라이브 API 플릿 (105 스위트·실 HTTP+psql 검증)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS 105/105</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>정적 게이트 6종 (테넌트/커서/동사/거버넌스/FK/잔재)</t>
+          <t>정적 게이트 7종 (테넌트/커서/동사/거버넌스/FK/잔재/i18n)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>P0/P1 요구사항 63/63 구현·검증 완료. 구현 스코프에서 launch 가능. 잔여는 사용자 결정·AI 크레딧 대기.</t>
+          <t>P0/P1 요구사항 63/63 구현·검증 완료. 동시성·자원고갈 하드닝 전면(9.16~9.22) + 마스터 대장 검색(9.23~9.25). 전 화면 60/60·플릿 105/105 실측. 구현 스코프에서 launch 가능. 잔여는 사용자 결정(#72~#80)·AI 크레딧 대기.</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3845,6 +3845,270 @@
       <c r="D14" s="2" t="inlineStr">
         <is>
           <t>라이브 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>9.14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>AI 질의 감사 추적</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>#64 ai_chat 감사(질문·참조·사용자)·alembic 0054 SECURITY 소스</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>라이브 6/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>9.15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Macro AI 무상태 불변식</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>#65 macro-generate 초안만 반환·게시 불가</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>라이브 7/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>9.16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>DB 풀 상향</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>min1/max4→min2/max12 (읽기 동시성 병목 해소)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>부하 재측정</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>9.17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>실시간 DB 부하 신호</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>/system/status dbLoad(활성쿼리·최장쿼리)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>라이브 9/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>9.18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>프로젝트 채번 경쟁 수정</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>동시 생성 500(12중7)→ON CONFLICT 재시도 전량 201</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>라이브 5/5</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>9.19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>채번기 5종 경쟁 안전화</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>eco/wo/qc/po/산출물 동일 버그 클래스 전수 제거</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>라이브 5/5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>9.20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>트랜잭션 그리드 안전 상한</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>무한성장 7종 최신순 limit 회로차단(OOM 방지)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>라이브 18/18</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>9.21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>내보내기 메모리 상한</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>export.xlsx 6종 LIMIT+절단 고지(공유 백엔드 OOM)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>라이브 20/20</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>9.22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>잔여 그리드 상한</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>anomalies·supplier-evals 상한 + 전 플릿 105/105</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>라이브 24/24</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>9.23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>마스터 검색: 부품·거래처</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>서버측 q 부분일치(ILIKE, 하위호환)·SearchBox</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>라이브 10/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>9.24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>마스터 검색: 자재·도면</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>동일 패턴 확장</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>라이브 17/17</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>9.25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>마스터 검색: 제품코드</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>대형 마스터 5종 전부 검색 가능</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>라이브 21/21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.38: fix(a11y): muted 텍스트 대비 WCAG AA 충족 — --txt-mute #8B93A1(3.09:1)→#626A7A(4.5+), Launch 시트6 조치완료
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -4435,12 +4435,12 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>설계 결정 필요</t>
+          <t>조치완료(9.38)</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>주 텍스트 15:1(우수). --txt-mute #8B93A1 ≈3.2:1 은 WCAG AA 일반텍스트(4.5:1) 미달·큰텍스트(3:1) 통과. 의도적 약화 텍스트라 darken 은 시각 위계 변경 — 디자인 소유자 판단</t>
+          <t>--txt-mute #8B93A1(3.09:1, AA 미달)→#626A7A 로 어둡게 — 흰색 5.44·회색패널 4.5+ 로 WCAG AA 충족, 텍스트 계층 유지</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.66: docs: 전 플릿 재검증 113/113 green 기록 — 신규 기능 5종 회귀 0·신규 라우트 성능 검증(dwg_file 2168행 조인 Index Scan 0.6ms)·Launch 요약 스위트 수 갱신(108→113)
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -629,12 +629,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>라이브 API 플릿 (108 스위트·실 HTTP+psql, 시드 자기치유)</t>
+          <t>라이브 API 플릿 (113 스위트·실 HTTP+psql, 시드 자기치유)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PASS 108/108</t>
+          <t>PASS 113/113</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>P0/P1 요구사항 63/63 구현·검증 완료. 동시성·자원고갈 하드닝 전면(9.16~9.22)·마스터/트랜잭션 검색(9.23~9.31) ·정보접근 마스킹 우회 차단(9.37)·i18n 62화면 파리티(3로케일)·접근성 4개 WCAG 축(대비/포커스/이름/키보드, 9.38~9.41). 전 화면 62/62·플릿 108/108 실측. 구현 스코프 launch 가능. 잔여는 사용자 결정(#72~#80)·AI 크레딧 대기.</t>
+          <t>P0/P1 요구사항 63/63 구현·검증 완료. 동시성·자원고갈 하드닝 전면(9.16~9.22)·마스터/트랜잭션 검색(9.23~9.31) ·정보접근 마스킹 우회 차단(9.37)·i18n 62화면 파리티(3로케일)·접근성 4개 WCAG 축(대비/포커스/이름/키보드, 9.38~9.41). 전 화면 62/62·플릿 113/113 실측. 구현 스코프 launch 가능. 잔여는 사용자 결정(#72~#80)·AI 크레딧 대기.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
15.5: docs+test: 테넌트 export 통제 회귀 고정 및 15.3~15.4 문서 반영
- live_cost_masking: 테넌트 export 검증 추가(47/47). set_mode 에 role 인자를 넣어
  **ADMIN 역할**에 제한을 걸도록 수정 — export 는 ADMIN 전용이라 GENERAL 에 걸면
  호출 자체가 403 이라 통제 여부를 확인할 수 없다(첫 시도에서 실제로 그렇게 빗나갔다).
  정리 블록에서 ADMIN 역할 제한도 되돌린다.
- 진행현황·Launch 하드닝 이력·보안 감사에 15.3~15.4 기록(실증 수치 포함:
  full 14파일 → no_download 13파일 → 복귀 시 재포함).
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3543,7 +3543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4957,6 +4957,28 @@
       <c r="D64" s="2" t="inlineStr">
         <is>
           <t>라이브 43/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>15.3~15.4</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>세션·알림·오프보딩</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>알림 읽음 거짓 성공 수정 + 비활성화 즉시 차단 회귀 고정 + 테넌트 export 의 금액 테이블 Export 통제 적용(제외 사실 고지)</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>라이브 18/18·47/47</t>
         </is>
       </c>
     </row>
@@ -4971,7 +4993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5439,6 +5461,28 @@
       <c r="D21" s="7" t="inlineStr">
         <is>
           <t>Excel Import 6곳이 파일 전체를 메모리로 읽고 있었다 — 공용 헬퍼로 20MB 상한·빈 파일 거부, 초과 시 413 에 크기 병기</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Export 통제</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>테넌트 오프보딩 export</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>조치완료(15.4)</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>금액 테이블(cst_quotation)이 Export 통제 없이 덤프됐다 — 해당 테이블만 제외하고 manifest·헤더·감사에 사유 기재(오프보딩 자체는 계약상 권리라 막지 않는다)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
18.0: docs: 승인 상태 기계 점검(17.1~17.9) 종합 반영 — 플릿 134/134
- 진행현황: 17.7·17.9 항목 추가, 17.1~17.2 의 플릿 수치 확정(134/134)
- Launch 준비 요약: 스위트 124 + 게이트 10종 = 134, 중간 배포 없는 깨끗한 실행
- 하드닝 이력 17.9 추가
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -629,12 +629,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>라이브 API 플릿 (121 스위트·실 HTTP+psql, 시드 자기치유·잔재 자가정리)</t>
+          <t>라이브 API 플릿 (124 스위트·실 HTTP+psql, 시드 자기치유 포함) + 정적/브라우저 게이트 10종</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PASS 132/132 (스위트 122 + 게이트 10종 · 중간 배포 없는 실행 · 2026-07-26)</t>
+          <t>PASS 134/134 (스위트 124 + 게이트 10종 · 중간 배포 없는 깨끗한 실행 · 2026-07-26). 승인 상태 기계 점검(17.1~17.9) 반영 — 상태 CHECK 제약, 승인 대상 소유 검증, 묵은 요청 차단 포함</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5221,6 +5221,28 @@
       <c r="D76" s="2" t="inlineStr">
         <is>
           <t>live_approval_tenant 8/8 — 타 테넌트 행 실재 확인 후 404</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>17.9</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>잔재 게이트 진단 안내 보강</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>플릿의 유일한 실패가 잔재 게이트였는데, 잔재 증가가 아니라 앞선 실패 실행이 남긴 값을 이번 실행이 정리한 것이었다(PENDING 1→0). live_all 이 스위트 직전에 기준 지문을 저장하므로 더러운 상태로 시작하면 잔재가 기준선에 들어간다. 0 으로 줄어든 항목은 그 가능성을 함께 안내.</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>DB 직접 확인 — F5T 0건 · 고아 승인요청 0건 · code_item_value 23건 전량 APPROVED. 깨끗한 상태 재실행 플릿 134/134</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
18.8: docs: 플릿 136/136 확정 반영 (게이트 12종)
중간 배포 없는 실행 — /health.proc 불변, 재시작 경고 0건, exit 0.
- Launch 준비 요약 14·15행: 게이트 12종·136/136 확정
- 하드닝 이력 18.6~18.7 추가
- 진행현황 머리표: 플릿 136/136 반영
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -629,24 +629,24 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>라이브 API 플릿 (124 스위트·실 HTTP+psql, 시드 자기치유 포함) + 정적/브라우저 게이트 11종</t>
+          <t>라이브 API 플릿 (124 스위트·실 HTTP+psql, 시드 자기치유 포함) + 정적/브라우저 게이트 12종</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PASS 135/135 (스위트 124 + 게이트 11종 · 2026-07-26). 중간 배포 없음을 러너가 스스로 확인한 실행 — /health.proc 이 시작·종료 시점에 동일(18.4). 승인 상태 기계(17.1~17.9)·인쇄리포트/Import (17.10~17.12)·DB정의서 생성 전환(18.2) 반영</t>
+          <t>PASS 136/136 (스위트 124 + 게이트 12종 · 2026-07-26). 중간 배포 없음을 러너가 확인한 실행(/health.proc 불변). 승인 상태 기계(17.1~17.9)·인쇄리포트/Import(17.10~17.12)·문서 생성 전환(18.2 DB정의서 · 18.6 API 계약) 반영</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>정적/브라우저 게이트 11종 (테넌트/커서/동사/거버넌스/DB정의서/FK/잔재/i18n 62화면/a11y 이름 62화면/감사 커버리지/검증 코드 문법·인자수)</t>
+          <t>정적/브라우저 게이트 12종 (테넌트/커서/동사/거버넌스/DB정의서/API계약/FK/잔재/i18n 62화면/a11y 이름 62화면/감사 커버리지/검증 코드 문법·인자수)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>ALL PASS — DB정의서 게이트는 18.2 신설(문서=생성기 + 스냅샷=실 스키마)</t>
+          <t>ALL PASS — DB정의서(18.2)·API계약(18.6) 게이트 신설</t>
         </is>
       </c>
     </row>
@@ -3593,7 +3593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5381,6 +5381,28 @@
       <c r="D81" s="2" t="inlineStr">
         <is>
           <t>플릿 135/135 · proc 불변 확인(재시작 경고 0건 · exit 0) — 러너가 스스로 '깨끗한 실행' 을 확인한 첫 결과</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>18.6~18.7</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>API 계약 as-built 전환 + 추적성 과대 주장 제거</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>컴포넌트정의서 API목록 108건 중 라우터에 그대로 있는 것은 42건(경로 상이 31·메서드 상이 9·미구현 26). 배포 app.openapi() 기준으로 생성 전환(446 오퍼레이션)하고 설계 초안은 대조 시트로 보존. 추적표 커버리지 '100%' 를 고리별 실측(요구사항→기능 100 · 기능→화면 55%)으로 교체. 구형 /api 라우터 5개는 앱 인증이 없고 nginx auth_basic 한 줄에만 의존하던 것을 불변식으로 고정.</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>플릿 136/136(게이트 12종) · live_security_headers 12→17 · check_api_contract 신설</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
18.12: docs: 18.9~18.11 반영 + 검증 경로 수정 (프로젝트 목록은 /projects)
- 진행현황: 18.9~18.10(결정성·커버리지 실측)·18.11(대화 절단) 항목
- 하드닝 이력 2건 · 위험대장 R-38(산출물 지문에 휘발성 값)
- 개발표준 2규약: "결정성은 깨질 조건을 일부러 만들어 확인한다" /
  "커버리지는 실행을 세고, 못 잰 것은 낮은 값으로 보고하지 않는다"
- live_project_comments: 프로젝트 목록 경로 오기 수정(/erp/projects → /projects). 20/20 통과

작업 메모: 문서 문장을 `py -c "…"` 로 삽입하면서 백틱이 bash 명령 치환으로 먹혀 본문 일부가
빈 칸으로 들어갔다(세션 중 세 번째 인용 사고 — 앞선 둘은 heredoc 의 \n 이었다). Edit 로
복구하고 백틱 짝·길이를 확인했다. 문서 본문 삽입은 Write/Edit 로 한다.
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3593,7 +3593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D83"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5425,6 +5425,28 @@
       <c r="D83" s="2" t="inlineStr">
         <is>
           <t>임계 실측(gap 1.0s 불일치 → 수정 후 0·1.0·2.5s 동일, 다른 파라미터는 여전히 다름) · 수정 전 배포본에서 검증 실패 확인 · live_drawing_job 18/18 · API 커버리지 419/446(93%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>18.11</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>수정 불가 대화의 조용한 절단 + 미검증 쓰기 경로 보강</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>API 표면 실측(18.9)에서 플릿이 한 번도 두드리지 않는 쓰기 경로 8건이 드러났다. 그중 프로젝트 대화 등록이 1000자에서 조용히 잘렸다 — 대화는 '수정 불가' 규약이라 되돌릴 수도 없고 사용자는 잃은 줄 모른다. 초과는 422 로 거부하고 실제 자수·상한을 사유에 담는다.</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>live_project_comments 20/20 — 상한 초과 422·사유의 자수·잘린 행 미생성·경계 1000자 통과 (과잉 차단 아님)·남의 글 GENERAL 403·ADMIN 삭제·삭제 감사에 원본 보존</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
18.13: docs: 플릿 137/137 · API 표면 커버리지 94% 확정 반영
중간 배포 없는 실행 — /health.proc 불변, 재시작 경고 0건, exit 0.
- Launch 준비 요약: 스위트 125 + 게이트 12종 = 137/137
- 요약에 'API 표면 커버리지(실측)' 행 신설 — 422/446(94%), 미호출 24
  (검증 소스의 경로 문자열이 아니라 실제 요청 로그를 센다)
- 진행현황 머리표에 커버리지 수치 추가
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -629,12 +629,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>라이브 API 플릿 (124 스위트·실 HTTP+psql, 시드 자기치유 포함) + 정적/브라우저 게이트 12종</t>
+          <t>라이브 API 플릿 (125 스위트·실 HTTP+psql, 시드 자기치유 포함) + 정적/브라우저 게이트 12종</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PASS 136/136 (스위트 124 + 게이트 12종 · 2026-07-26). 중간 배포 없음을 러너가 확인한 실행(/health.proc 불변). 승인 상태 기계(17.1~17.9)·인쇄리포트/Import(17.10~17.12)·문서 생성 전환(18.2 DB정의서 · 18.6 API 계약) 반영</t>
+          <t>PASS 137/137 (스위트 125 + 게이트 12종 · 2026-07-26). 중간 배포 없음을 러너가 확인(/health.proc 불변). 승인 상태 기계(17.1~17.9)·인쇄리포트/Import(17.10~17.12)·문서 생성 전환(18.2·18.6)·산출물 결정성(18.10)·대화 절단(18.11) 반영</t>
         </is>
       </c>
     </row>
@@ -687,16 +687,28 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="2" t="inlineStr"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>API 표면 커버리지 (실측 — 요청 로그 기준)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>422/446 (94%) · 미호출 24건 (구형 /api 5 · 읽기 전용 다수). 검증 소스의 경로 문자열이 아니라 실제 호출을 센다</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>판정</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>P0/P1 요구사항 63/63 구현·검증 완료. 동시성·자원고갈 하드닝(9.16~9.22)·마스터/트랜잭션 검색(9.23~9.31)·정보접근 마스킹 우회 차단(9.37)·i18n 62화면 파리티(3로케일)·접근성 4개 WCAG 축(9.38~9.41). 2026-07-26 구간에서 인증 하드닝 3건(세션 서명키 기본값·비밀번호 해시·복구 경로)과 운영 데이터 실결함 4건(단가 미해결이 견적을 낮추던 경로·업무 날짜 하루 밀림·계층 이동 손상·토큰 서명키)을 실측 근거와 함께 해소했고, 규격 미구현 3건(CPQ-001 제품 선택·DOC-001 문서 개정·ADM-003 승인 위임)을 구현했다. 전 화면 62/62 · 플릿 131/131(스위트 121 + 게이트 10종) 실측. 구현 스코프 launch 가능. 잔여는 사용자 결정(#72~#80)·AI 크레딧 대기·감사 커버리지 7건(게이트로 증가 차단, 위험 순 축소 중).</t>
         </is>

</xml_diff>

<commit_message>
18.18: docs: 플릿 138/138 확정 반영 (스위트 126 + 게이트 12종)
중간 배포 없는 실행 — /health.proc 불변, 재시작 경고 0건, exit 0.
Launch 준비 요약·진행현황 머리표 갱신.
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -629,12 +629,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>라이브 API 플릿 (125 스위트·실 HTTP+psql, 시드 자기치유 포함) + 정적/브라우저 게이트 12종</t>
+          <t>라이브 API 플릿 (126 스위트·실 HTTP+psql, 시드 자기치유 포함) + 정적/브라우저 게이트 12종</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PASS 137/137 (스위트 125 + 게이트 12종 · 2026-07-26). 중간 배포 없음을 러너가 확인(/health.proc 불변). 승인 상태 기계(17.1~17.9)·인쇄리포트/Import(17.10~17.12)·문서 생성 전환(18.2·18.6)·산출물 결정성(18.10)·대화 절단(18.11) 반영</t>
+          <t>PASS 138/138 (스위트 126 + 게이트 12종 · 2026-07-26). 중간 배포 없음을 러너가 확인(/health.proc 불변). 승인 상태 기계(17.1~17.9)·인쇄리포트/Import(17.10~17.12)·문서 생성 전환(18.2·18.6)·산출물 결정성(18.10)·대화 절단(18.11)·목록 절단 고지(18.14)·삭제 이력 보존(18.16) 반영</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
18.26: docs: 18.25 반영 — R-39 누적 25/34, 잔여 9곳 후순위 근거 기재
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3605,7 +3605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D89"/>
+  <dimension ref="A1:D90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5569,6 +5569,28 @@
       <c r="D89" s="2" t="inlineStr">
         <is>
           <t>live_delete_history 17→20 — 매크로 수식(=A*2+7)·상태·버전·참조 삭제 건수 보존 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>18.25</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>삭제 이력 보존 — 부품·창고·Templet·견적안</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>부품은 번호만 남기고 이름·규격과 함께 지운 공급자 코드 매핑 건수(조달 경로)가 없었다. 견적안은 완성품 코드만 남겼는데 슬롯 선택값이 곧 그 견적안의 내용이다(같은 코드라도 슬롯이 다르면 다른 제품). 창고·Templet 도 이름/코드만 있었다. 넷 다 after 를 before 로 바로잡고 DELETE 에 테넌트 조건 추가(기준선 64→62).</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>live_delete_history 20→23 — 창고 이름·유형 보존 확인</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
18.42: docs: 18.41 반영 — R-41 누적 11종, 잔여 15곳
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3605,7 +3605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5745,6 +5745,28 @@
       <c r="D97" s="2" t="inlineStr">
         <is>
           <t>live_cad_blocks 8/8 신설 — 상한 초과 422·사유의 개수(501)/상한(500)·경계값 500 통과·.dxf 응답이 실제 DXF</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>18.41</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>수정 이력 — 프로젝트 단계·Contract 선언</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>영업 단계 전이는 사업 진행 상태 그 자체이고 납기일 변경은 일정 약속이 바뀐 것인데 새 값만 남았다. 바뀐 필드만 before 에 담는다(안 바꾼 값까지 넣으면 대조가 흐려진다). Contract 는 '어떤 원천의 어떤 필드를 쓸 수 있는지' 선언하는 통제라 이전 선언이 남아야 허용 필드 증가를 확인할 수 있다 — 신규 등록은 before 에 그 사실을 명시해 빈 값과 구분.</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>live_delete_history 30→32 — 프로젝트 수정 이력에 이전 값 보존. 기준선 62→61</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.48: fix: 모르는 필터 값을 조용히 버리던 3곳 422(18.62), GC 의 교차 테넌트 삭제 차단(18.63) — live_filter_honesty 신규·live_storage_ns 확장
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3605,7 +3605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D109"/>
+  <dimension ref="A1:D111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6009,6 +6009,50 @@
       <c r="D109" s="2" t="inlineStr">
         <is>
           <t>18.59 이전 상태 사본에서 edim.py::project_files::project 탐지 확인 · 현재 기준선 0항목</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>18.62</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>모르는 필터 값을 조용히 버리던 3곳 — 빈 값과 모르는 값을 구분</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>/anomalies(status·source)는 모르는 값이면 조건을 붙이지 않고 전체를 돌려줬고, /arrangements(forCode)는 없는 코드를 '제품군 없음'으로 스코프했으며, /cost/variance(project)는 없는 프로젝트에 0 분석표를 돌려줬다. 빈 값=전체 보기는 유지하고 모르는 값만 422.</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>필터 GET 63개 중 48건 실측(4건 동일 → 3건 결함) · live_filter_honesty 신규(고친 3곳 + 필터 25쌍 광역 회귀, 건너뛴 건수 출력)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>18.63</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>GC 가 다른 테넌트의 객체를 지울 수 있던 문제</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>/files/gc 는 테넌트 ADMIN 권한인데 버킷은 공유다. 18.57 이전엔 소유를 판별할 단서가 없어 전역으로 훑었고, 이제 t{tid}/ 접두사가 있으므로 남의 접두사 객체는 대상에서 뺀다. 접두사 없는 옛 객체는 종전대로 둔다(없는 근거로 지우거나 남기지 않는다). foreignSkipped 로 몇 건을 뺐는지 응답에 드러낸다.</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>수정 전 실증 — t9999/ 프로브 객체를 orphan 1건으로 잡고 sampleOrphans 에 노출(apply=true 면 삭제) → 수정 후 orphans 0·foreignSkipped 1 (live_storage_ns)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.52: fix: MRP 재고 대조 불가를 '보유 0'과 구분(18.73) — UNMATCHED 상태·미대조 건수 노출, live_mrp_match 신규
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3590,7 +3590,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>추적표 화면 ID 는 W-01 계열, 구현은 C-1·D-1 계열 · 메뉴 기능코드는 E-x·S-x-x, 구현 화면코드와 일치 26/89 · API 경로도 설계 108건 중 42건만 일치. 어느 쪽을 기준으로 삼을지(또는 매핑표를 확정할지) 결정 필요 — 추측으로 이으면 그럴듯한 오답이 된다. 결정 전까지 REQ→기능→메뉴→화면→컴포넌트→DB 사슬은 화면 이후가 코드로 이어지지 않는다</t>
+          <t>추적표 화면 ID 는 W-01 계열, 구현은 C-1·D-1 계열 · 메뉴 기능코드는 E-x·S-x-x, 구현 화면코드와 일치 26/89 · API 경로도 설계 108건 중 42건만 일치. 어느 쪽을 기준으로 삼을지(또는 매핑표를 확정할지) 결정 필요 — 추측으로 이으면 그럴듯한 오답이 된다. 결정 전까지 REQ→기능→메뉴→화면→컴포넌트→DB 사슬은 화면 이후가 코드로 이어지지 않는다 · **영향 실측(18.73)**: 수주 라인은 변형 코드(ECC 55-32), 마스터·재고는 기준 코드(ECC 55)라 MRP 재고 대조가 수요 8건 전부 실패 → 계획이 늘 '전 품목 발주 필요'로 나온다. 구매요청 화면(/erp/pr-items)도 이 결정 전에는 실수요로 전환할 수 없어 데모 3건 고정이다.</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D120"/>
+  <dimension ref="A1:D121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6251,6 +6251,28 @@
       <c r="D120" s="2" t="inlineStr">
         <is>
           <t>seed_heal 로 BOM 4행 원복 · 잔존 프로브 부품 삭제 · check_live_residue 22항목 지문 일치</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>18.73</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>MRP 재고 대조 불가를 '보유 0'으로 보고하던 문제</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>수주 라인은 변형 코드(ECC 55-32), 마스터·재고는 기준 코드(ECC 55)라 on_hand.get(code,0) 이 늘 0 이 됐다. 실측: 수요 8건 전부 보유 0·부족 8건인데 창고에는 실재고 존재. 코드 매칭 규칙은 식별자 체계 결정(#81) 사안이라 정하지 않고, 대조 불가를 UNMATCHED(onHand·shortage=null)로 구분해 건수를 응답·화면에 노출.</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>운영 실측 8/8 미대조 확인 · tsc 통과 · MrpGrid 대조불가 칩·컬럼 '—' 표기</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.60: docs: 18.76 묶음 상한·누락 고지 기록 + live_zip_bounds 플릿 등록
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3605,7 +3605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D123"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6317,6 +6317,28 @@
       <c r="D123" s="2" t="inlineStr">
         <is>
           <t>배포본 Playwright 재확인에서 발견 · tsc 통과 · 구매/PCR 화면 표기 교정</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>18.76</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>파일 묶음 상한 부재·누락 무고지 해소</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>/files/zip 은 미호출 경로였다. 프로젝트 하나가 4,990건·79MB 인데 상한 없이 메모리에서 압축했고, 저장소에서 못 받은 객체는 조용히 건너뛰며 아무것도 알리지 않았다. 상한(1,000건·200MB) 초과는 잘라 주지 않고 413 거부(사유에 실제 규모·분할 안내), 누락은 X-Missing 헤더와 묶음 안 _누락파일.txt 로 고지. 고객 전달본도 동일 상한.</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>live_zip_bounds 14/14 신규 — 전체 413 · DATA 폴더 200 · 없는 객체 행 삽입 시 X-Missing 1·누락 메모·파일명 확인</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.70: test: Project Folder 상한·현재 Run 구분 회귀 추가 + 18.82 문서 반영
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3627,7 +3627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D129"/>
+  <dimension ref="A1:D130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6471,6 +6471,28 @@
       <c r="D129" s="2" t="inlineStr">
         <is>
           <t>live_zip_bounds 23/23 — 헤더·매니페스트 일치, 기준 Run is_test=f, 담긴 산출물 중 테스트 Run 0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>18.82</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Project Folder 목록 상한·절단 고지 + 현재 Run 구분</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>업로드 구간 쿼리에 LIMIT 이 없어 한 프로젝트 5,156행을 매 조회마다 전량 전송했다(Run 마다 증가). 상한 500 + X-Truncated/X-Limit 헤더와 화면 상한 칩 적용. 아울러 지난 Run 산출물이 현재 납품물과 같은 '산출물' 표기로 섞여 구분되지 않던 것을 run·currentRun 노출과 '현재' 칩으로 해소.</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>실측 5,156행 → 503행(500+최신 Run 3) · X-Truncated true · 현재 Run 3건만 표시 · live_storage_ns 36/36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.78: test: Project Folder 숨김·절단 화면 표시 회귀 추가 + 18.84 문서 반영
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3627,7 +3627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D131"/>
+  <dimension ref="A1:D132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6515,6 +6515,28 @@
       <c r="D131" s="2" t="inlineStr">
         <is>
           <t>PS-61313-5 73행(숨김 5,163)·PS-598 216행·PS-612 0행 · allRuns=true 1,000행 절단 고지 · live_f1_project 30/30 · live_storage_ns 36/36</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>18.84</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>숨김·절단 사실을 화면까지 전달</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>18.83 의 숨김 건수를 헤더로만 알려 화면에 닿지 않았다(18.79 와 같은 실수를 내 변경에 반복). apiServer 가 헤더를 버리는 구조라 SSR 이 접근할 수 없었던 것이 원인 — apiServerWith 추가. Project Folder 에 '지난 Run 산출물 숨김 N' 칩·전체/현재 Run 전환·'표시 상한 도달' 칩 표시.</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>기본 73건+숨김 5,202 표시 · 전체 1000건+상한 칩 · JS 오류 0 · live_storage_ns 40/40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.85: test: 감사 facet 비용 회귀 추가 + 18.87 문서 반영
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3649,7 +3649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D134"/>
+  <dimension ref="A1:D135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6603,6 +6603,28 @@
       <c r="D134" s="2" t="inlineStr">
         <is>
           <t>테이블·객체 크기, 일자별 증가, 동작별 분포 실측 · 위험 R-51 · 증가율은 검증 트래픽이 대부분이라 운영 예측치 아님을 명시</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>18.87</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>감사 조회 facet 의 전수 스캔 제거 (본 조회의 100배 비용)</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>본 조회는 인덱스로 0.6ms 인데 필터 드롭다운 두 질의가 Seq Scan(action 49.8ms·login_id 61.8ms, 105,639행)이었다. 사용자 목록은 사용자 대장에서 얻고, 동작 목록은 alembic 0063 인덱스 + loose index scan(재귀 CTE)으로 행 수가 아닌 값 종류에 비례하게 바꿈(33.7ms→1.7ms).</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>EXPLAIN ANALYZE 실측 · live_run_retention 14/14(Seq Scan 부재·인덱스 사용·사용자 출처 확인)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.90: docs: 18.91 오프보딩 export 보강 기록
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3693,7 +3693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D138"/>
+  <dimension ref="A1:D139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6735,6 +6735,28 @@
       <c r="D138" s="2" t="inlineStr">
         <is>
           <t>archive_mode/wal_level·버킷 versioning 실측 · RPO 24h 충족·복원 실측 30초로 RTO 여유 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>18.91</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>오프보딩 export 에 제품 구성 자산 추가 (13→22종)</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Code Set-up 마스터(code_group·code_item·code_item_value)가 통째로 빠져 제품 코드는 나가는데 그 코드를 만드는 규칙은 나가지 않았다. BOM·단가·Macro·치수·Arrangement·파일 목록도 부재. 9종 추가(dwg_bom 은 도면 경유로 테넌트 좁힘, 단가는 cost 통제 유지), 매니페스트에 파일 원본 채널과 files.json 대조표 안내 추가.</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>live_tenant_export 20/20 신규 — 포함 여부·DB 건수 일치(code_groups 3·values 23·macros 7·files 5,659)·민감 필드 부재·통제 시 단가만 제외 확인</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9.94: docs: 18.94 PCR 감사 누락 기록
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3697,7 +3697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D141"/>
+  <dimension ref="A1:D142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6805,6 +6805,28 @@
       <c r="D141" s="2" t="inlineStr">
         <is>
           <t>live_mfa 14/14 신규 — 전용 프로브 계정 생성·삭제(실 계정 잠금 방지) · TOTP 를 검증 측에서 독립 구현해 서버 구현과 대조</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>18.94</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>PCR 생성·수정 감사 누락 해소 (예외 목록 7→6)</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>감사 예외 목록이 '금액·판단 근거에서 한 단계 떨어져 있다'는 한 줄 사유 아래 POST /cost/pcr 를 담고 있었으나 PCR 은 견적 확정의 근거 금액이다. cst_pcr 이력 132건이 전부 MASKED_READ 로, 변경 기록이 전무했다. upsert 전 이전 값을 읽어 before/after 로 남기고 금액의 근거(기준 Run·테스트 여부·미해결 건수·마진율)를 함께 기록.</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>배포 후 실측 — UPDATE 이력에 before(직접원가·기여마진·EBIT·상태)·after(+basisRunId·basisIsTest·unpricedCount) 확인 · 게이트 기준선 6건</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
10.16: docs: DB 정의서·딜리버러블에 19.7 반영 (code_relationship.approved_basis_hash)
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_Launch준비상태.xlsx
@@ -3700,7 +3700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D154"/>
+  <dimension ref="A1:D155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7094,6 +7094,28 @@
       <c r="D154" s="11" t="inlineStr">
         <is>
           <t>live_ai_prep 27/27·live_security_anomaly 13/13 재실행 후 잔재 0 · 기존 993행(+감사 5행) 제거, 운영 테넌트 무영향</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="11" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="B155" s="11" t="inlineStr">
+        <is>
+          <t>승인 당시 전개 근거 지문 + basisDrift (#35)</t>
+        </is>
+      </c>
+      <c r="C155" s="11" t="inlineStr">
+        <is>
+          <t>승인된 관계는 삭제가 막히는데(DRAFT 한정) 슬롯 매핑은 자유롭게 바뀌었다 — 매핑은 BOM 전개의 유일한 근거이므로 승인 이후 바뀌면 승인된 내용과 현재 내용이 다른데 화면은 APPROVED 만 보여 줬다. 승인 시점 지문(approved_basis_hash, alembic 0064)을 남기고 현재 지문과 다르면 basisDrift 로 노출. 횟수가 아니라 내용 비교라 되돌리면 드리프트가 사라진다. 기존 승인 관계 14건은 backfill 로 오탐 방지.</t>
+        </is>
+      </c>
+      <c r="D155" s="11" t="inlineStr">
+        <is>
+          <t>live_slot_map 19→22 (드리프트 발생·복원 시 소멸·필드 노출) · DB 정의서 컬럼 1190→1191 갱신</t>
         </is>
       </c>
     </row>

</xml_diff>